<commit_message>
data: manual full refresh 2026-07-08
Reran all 35 state scrapers. 27 states advanced; LA/NJ/TN/WV/MT reached
June 2026, most others reached May 2026. KY refreshed Mar->May via the new
Tableau bootstrapSession scraper. Master workbooks rebuilt through Jun 2026.
DC/NH could not refresh locally (corporate TLS proxy blocks those domains);
to be picked up on the VPS.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/OSB_Master_Handle_GGR_Hold.xlsx
+++ b/data/processed/OSB_Master_Handle_GGR_Hold.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Handle'!$A$1:$CY$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'GGR'!$A$1:$CY$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hold'!$A$1:$CY$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Handle'!$A$1:$CZ$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'GGR'!$A$1:$CZ$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hold'!$A$1:$CZ$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CY37"/>
+  <dimension ref="A1:CZ37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -602,6 +602,7 @@
     <col width="12" customWidth="1" min="101" max="101"/>
     <col width="12" customWidth="1" min="102" max="102"/>
     <col width="12" customWidth="1" min="103" max="103"/>
+    <col width="12" customWidth="1" min="104" max="104"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1118,6 +1119,11 @@
       <c r="CY1" s="1" t="inlineStr">
         <is>
           <t>May 2026</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
         </is>
       </c>
     </row>
@@ -1375,6 +1381,7 @@
       <c r="CY2" s="4" t="n">
         <v>113140840</v>
       </c>
+      <c r="CZ2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1598,6 +1605,7 @@
         <v>737163558.23</v>
       </c>
       <c r="CY3" s="4" t="n"/>
+      <c r="CZ3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1852,7 +1860,10 @@
       <c r="CX4" s="4" t="n">
         <v>521196658.12</v>
       </c>
-      <c r="CY4" s="4" t="n"/>
+      <c r="CY4" s="4" t="n">
+        <v>469087369.44</v>
+      </c>
+      <c r="CZ4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2078,6 +2089,7 @@
       <c r="CY5" s="4" t="n">
         <v>188021266</v>
       </c>
+      <c r="CZ5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2327,6 +2339,7 @@
       <c r="CY6" s="4" t="n">
         <v>67182047.59</v>
       </c>
+      <c r="CZ6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2462,6 +2475,7 @@
       <c r="CY7" s="4" t="n">
         <v>18185343</v>
       </c>
+      <c r="CZ7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2739,6 +2753,7 @@
       <c r="CY8" s="4" t="n">
         <v>191112433.58</v>
       </c>
+      <c r="CZ8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2998,6 +3013,7 @@
         <v>1200999825.68</v>
       </c>
       <c r="CY9" s="4" t="n"/>
+      <c r="CZ9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3273,6 +3289,7 @@
       <c r="CY10" s="4" t="n">
         <v>428197306.01</v>
       </c>
+      <c r="CZ10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3462,6 +3479,7 @@
       <c r="CY11" s="4" t="n">
         <v>168118289</v>
       </c>
+      <c r="CZ11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3635,8 +3653,13 @@
       <c r="CW12" s="4" t="n">
         <v>300056064</v>
       </c>
-      <c r="CX12" s="4" t="n"/>
-      <c r="CY12" s="4" t="n"/>
+      <c r="CX12" s="4" t="n">
+        <v>230061384</v>
+      </c>
+      <c r="CY12" s="4" t="n">
+        <v>240541177</v>
+      </c>
+      <c r="CZ12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3859,7 +3882,10 @@
       <c r="CX13" s="4" t="n">
         <v>324485986.53</v>
       </c>
-      <c r="CY13" s="4" t="n"/>
+      <c r="CY13" s="4" t="n">
+        <v>317974369.23</v>
+      </c>
+      <c r="CZ13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4052,7 +4078,10 @@
       <c r="CX14" s="4" t="n">
         <v>678382514.61</v>
       </c>
-      <c r="CY14" s="4" t="n"/>
+      <c r="CY14" s="4" t="n">
+        <v>632109678.53</v>
+      </c>
+      <c r="CZ14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4274,6 +4303,7 @@
       <c r="CY15" s="4" t="n">
         <v>535415353.32</v>
       </c>
+      <c r="CZ15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4447,6 +4477,7 @@
       <c r="CY16" s="4" t="n">
         <v>40970519.45</v>
       </c>
+      <c r="CZ16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4690,6 +4721,7 @@
       <c r="CY17" s="4" t="n">
         <v>464796515.88</v>
       </c>
+      <c r="CZ17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4812,7 +4844,10 @@
       <c r="CX18" s="4" t="n">
         <v>273397862.9</v>
       </c>
-      <c r="CY18" s="4" t="n"/>
+      <c r="CY18" s="4" t="n">
+        <v>256364813.81</v>
+      </c>
+      <c r="CZ18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5110,6 +5145,7 @@
       <c r="CY19" s="4" t="n">
         <v>17298052.13</v>
       </c>
+      <c r="CZ19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5259,6 +5295,7 @@
       <c r="CY20" s="4" t="n">
         <v>4814407</v>
       </c>
+      <c r="CZ20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5426,6 +5463,7 @@
       <c r="CY21" s="4" t="n">
         <v>578070325</v>
       </c>
+      <c r="CZ21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5539,6 +5577,7 @@
       <c r="CW22" s="4" t="n"/>
       <c r="CX22" s="4" t="n"/>
       <c r="CY22" s="4" t="n"/>
+      <c r="CZ22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5808,6 +5847,7 @@
       <c r="CY23" s="4" t="n">
         <v>60919268</v>
       </c>
+      <c r="CZ23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6099,6 +6139,9 @@
       <c r="CY24" s="4" t="n">
         <v>912899287</v>
       </c>
+      <c r="CZ24" s="4" t="n">
+        <v>912899287</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6407,7 +6450,10 @@
       <c r="CX25" s="4" t="n">
         <v>922727272.73</v>
       </c>
-      <c r="CY25" s="4" t="n"/>
+      <c r="CY25" s="4" t="n">
+        <v>955592366.64</v>
+      </c>
+      <c r="CZ25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6627,6 +6673,7 @@
       <c r="CY26" s="4" t="n">
         <v>2132772287</v>
       </c>
+      <c r="CZ26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6808,18 +6855,19 @@
         <v>952964339</v>
       </c>
       <c r="CU27" s="4" t="n">
-        <v>929169341</v>
+        <v>812611457</v>
       </c>
       <c r="CV27" s="4" t="n">
-        <v>766738026</v>
+        <v>335614561</v>
       </c>
       <c r="CW27" s="4" t="n">
-        <v>663055400</v>
+        <v>352995396</v>
       </c>
       <c r="CX27" s="4" t="n">
-        <v>800138386</v>
+        <v>797769455</v>
       </c>
       <c r="CY27" s="4" t="n"/>
+      <c r="CZ27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7085,6 +7133,7 @@
       <c r="CY28" s="4" t="n">
         <v>77612245</v>
       </c>
+      <c r="CZ28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7120,13 +7169,13 @@
         <v>23353182.98</v>
       </c>
       <c r="Q29" s="4" t="n">
-        <v>32625607.32</v>
+        <v>35303747.82</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>28609318.09</v>
+        <v>28848348.27</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>28009704.96</v>
+        <v>28583539.15</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>39281991.12</v>
@@ -7380,6 +7429,7 @@
       <c r="CY29" s="4" t="n">
         <v>595569801.5</v>
       </c>
+      <c r="CZ29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7671,6 +7721,7 @@
       </c>
       <c r="CX30" s="4" t="n"/>
       <c r="CY30" s="4" t="n"/>
+      <c r="CZ30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7863,7 +7914,10 @@
       <c r="CX31" s="4" t="n">
         <v>596884.16</v>
       </c>
-      <c r="CY31" s="4" t="n"/>
+      <c r="CY31" s="4" t="n">
+        <v>491137.73</v>
+      </c>
+      <c r="CZ31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8110,6 +8164,9 @@
       </c>
       <c r="CY32" s="4" t="n">
         <v>443038330</v>
+      </c>
+      <c r="CZ32" s="4" t="n">
+        <v>456129258</v>
       </c>
     </row>
     <row r="33">
@@ -8352,6 +8409,7 @@
         <v>613893171</v>
       </c>
       <c r="CY33" s="4" t="n"/>
+      <c r="CZ33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8523,6 +8581,7 @@
       <c r="CY34" s="4" t="n">
         <v>13986635</v>
       </c>
+      <c r="CZ34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8779,6 +8838,9 @@
       </c>
       <c r="CY35" s="4" t="n">
         <v>32963899.18</v>
+      </c>
+      <c r="CZ35" s="4" t="n">
+        <v>5293841.94</v>
       </c>
     </row>
     <row r="36">
@@ -8836,26 +8898,54 @@
       <c r="AR36" s="4" t="n"/>
       <c r="AS36" s="4" t="n"/>
       <c r="AT36" s="4" t="n"/>
-      <c r="AU36" s="4" t="n"/>
-      <c r="AV36" s="4" t="n"/>
-      <c r="AW36" s="4" t="n"/>
+      <c r="AU36" s="4" t="n">
+        <v>6239052.17</v>
+      </c>
+      <c r="AV36" s="4" t="n">
+        <v>10847657.2</v>
+      </c>
+      <c r="AW36" s="4" t="n">
+        <v>10973008.49</v>
+      </c>
       <c r="AX36" s="4" t="n">
         <v>12285011.5</v>
       </c>
-      <c r="AY36" s="4" t="n"/>
+      <c r="AY36" s="4" t="n">
+        <v>13977632.49</v>
+      </c>
       <c r="AZ36" s="4" t="n">
         <v>10301603.38</v>
       </c>
-      <c r="BA36" s="4" t="n"/>
-      <c r="BB36" s="4" t="n"/>
-      <c r="BC36" s="4" t="n"/>
-      <c r="BD36" s="4" t="n"/>
-      <c r="BE36" s="4" t="n"/>
-      <c r="BF36" s="4" t="n"/>
-      <c r="BG36" s="4" t="n"/>
-      <c r="BH36" s="4" t="n"/>
-      <c r="BI36" s="4" t="n"/>
-      <c r="BJ36" s="4" t="n"/>
+      <c r="BA36" s="4" t="n">
+        <v>12704938.11</v>
+      </c>
+      <c r="BB36" s="4" t="n">
+        <v>9995919.880000001</v>
+      </c>
+      <c r="BC36" s="4" t="n">
+        <v>9340833.460000001</v>
+      </c>
+      <c r="BD36" s="4" t="n">
+        <v>7322852.34</v>
+      </c>
+      <c r="BE36" s="4" t="n">
+        <v>7246352.46</v>
+      </c>
+      <c r="BF36" s="4" t="n">
+        <v>10990903.54</v>
+      </c>
+      <c r="BG36" s="4" t="n">
+        <v>13575173.24</v>
+      </c>
+      <c r="BH36" s="4" t="n">
+        <v>17275316.71</v>
+      </c>
+      <c r="BI36" s="4" t="n">
+        <v>16702866.74</v>
+      </c>
+      <c r="BJ36" s="4" t="n">
+        <v>15087738.75</v>
+      </c>
       <c r="BK36" s="4" t="n">
         <v>14339351.38</v>
       </c>
@@ -8979,6 +9069,7 @@
       <c r="CY36" s="4" t="n">
         <v>16886244.07</v>
       </c>
+      <c r="CZ36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -9034,13 +9125,13 @@
         <v>848147571.8200001</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>1057833223.16</v>
+        <v>1060511363.66</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>706498673.59</v>
+        <v>706737703.77</v>
       </c>
       <c r="S37" s="6" t="n">
-        <v>700669103.42</v>
+        <v>701242937.61</v>
       </c>
       <c r="T37" s="6" t="n">
         <v>664509969.48</v>
@@ -9124,52 +9215,52 @@
         <v>3441006569.64</v>
       </c>
       <c r="AU37" s="6" t="n">
-        <v>5761127148.8</v>
+        <v>5767366200.97</v>
       </c>
       <c r="AV37" s="6" t="n">
-        <v>7948172773.95</v>
+        <v>7959020431.15</v>
       </c>
       <c r="AW37" s="6" t="n">
-        <v>7838641714.24</v>
+        <v>7849614722.73</v>
       </c>
       <c r="AX37" s="6" t="n">
         <v>7819711507.69</v>
       </c>
       <c r="AY37" s="6" t="n">
-        <v>10238345148.99</v>
+        <v>10252322781.48</v>
       </c>
       <c r="AZ37" s="6" t="n">
         <v>8224766760.92</v>
       </c>
       <c r="BA37" s="6" t="n">
-        <v>9562144401.42</v>
+        <v>9574849339.530001</v>
       </c>
       <c r="BB37" s="6" t="n">
-        <v>7725486044.51</v>
+        <v>7735481964.39</v>
       </c>
       <c r="BC37" s="6" t="n">
-        <v>6806759569.1</v>
+        <v>6816100402.56</v>
       </c>
       <c r="BD37" s="6" t="n">
-        <v>5249889332.85</v>
+        <v>5257212185.19</v>
       </c>
       <c r="BE37" s="6" t="n">
-        <v>4748832129.69</v>
+        <v>4756078482.15</v>
       </c>
       <c r="BF37" s="6" t="n">
-        <v>5103770537.47</v>
+        <v>5114761441.01</v>
       </c>
       <c r="BG37" s="6" t="n">
-        <v>8051643777.05</v>
+        <v>8065218950.29</v>
       </c>
       <c r="BH37" s="6" t="n">
-        <v>9879890119.93</v>
+        <v>9897165436.639999</v>
       </c>
       <c r="BI37" s="6" t="n">
-        <v>10134020423.52</v>
+        <v>10150723290.26</v>
       </c>
       <c r="BJ37" s="6" t="n">
-        <v>9621865638.77</v>
+        <v>9636953377.52</v>
       </c>
       <c r="BK37" s="6" t="n">
         <v>11483979710.59</v>
@@ -9280,23 +9371,26 @@
         <v>16396740854.21</v>
       </c>
       <c r="CU37" s="6" t="n">
-        <v>16279384890.64</v>
+        <v>16162827006.64</v>
       </c>
       <c r="CV37" s="6" t="n">
-        <v>13069231093.13</v>
+        <v>12638107628.13</v>
       </c>
       <c r="CW37" s="6" t="n">
-        <v>15435754952.1</v>
+        <v>15125694948.1</v>
       </c>
       <c r="CX37" s="6" t="n">
-        <v>13562654446.5</v>
+        <v>13790346899.5</v>
       </c>
       <c r="CY37" s="6" t="n">
-        <v>7101970694.71</v>
+        <v>9974131607.09</v>
+      </c>
+      <c r="CZ37" s="6" t="n">
+        <v>1374322386.94</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CY36"/>
+  <autoFilter ref="A1:CZ36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9307,7 +9401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CY37"/>
+  <dimension ref="A1:CZ37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9413,6 +9507,7 @@
     <col width="12" customWidth="1" min="101" max="101"/>
     <col width="12" customWidth="1" min="102" max="102"/>
     <col width="12" customWidth="1" min="103" max="103"/>
+    <col width="12" customWidth="1" min="104" max="104"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -9929,6 +10024,11 @@
       <c r="CY1" s="1" t="inlineStr">
         <is>
           <t>May 2026</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
         </is>
       </c>
     </row>
@@ -10186,6 +10286,7 @@
       <c r="CY2" s="4" t="n">
         <v>11314084</v>
       </c>
+      <c r="CZ2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -10409,6 +10510,7 @@
         <v>82599231.73</v>
       </c>
       <c r="CY3" s="4" t="n"/>
+      <c r="CZ3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -10663,7 +10765,10 @@
       <c r="CX4" s="4" t="n">
         <v>49863057.43</v>
       </c>
-      <c r="CY4" s="4" t="n"/>
+      <c r="CY4" s="4" t="n">
+        <v>44653912.41</v>
+      </c>
+      <c r="CZ4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -10889,6 +10994,7 @@
       <c r="CY5" s="4" t="n">
         <v>19242863</v>
       </c>
+      <c r="CZ5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -11138,6 +11244,7 @@
       <c r="CY6" s="4" t="n">
         <v>7672938.32</v>
       </c>
+      <c r="CZ6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -11273,6 +11380,7 @@
       <c r="CY7" s="4" t="n">
         <v>2028987</v>
       </c>
+      <c r="CZ7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -11548,6 +11656,7 @@
       <c r="CY8" s="4" t="n">
         <v>20785834.86</v>
       </c>
+      <c r="CZ8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -11805,6 +11914,7 @@
         <v>124797340.84</v>
       </c>
       <c r="CY9" s="4" t="n"/>
+      <c r="CZ9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -12080,6 +12190,7 @@
       <c r="CY10" s="4" t="n">
         <v>50167277.32</v>
       </c>
+      <c r="CZ10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -12269,6 +12380,7 @@
       <c r="CY11" s="4" t="n">
         <v>12339200</v>
       </c>
+      <c r="CZ11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -12442,8 +12554,13 @@
       <c r="CW12" s="4" t="n">
         <v>28909718</v>
       </c>
-      <c r="CX12" s="4" t="n"/>
-      <c r="CY12" s="4" t="n"/>
+      <c r="CX12" s="4" t="n">
+        <v>27187385</v>
+      </c>
+      <c r="CY12" s="4" t="n">
+        <v>26499056</v>
+      </c>
+      <c r="CZ12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -12664,7 +12781,10 @@
       <c r="CX13" s="4" t="n">
         <v>45844177.7</v>
       </c>
-      <c r="CY13" s="4" t="n"/>
+      <c r="CY13" s="4" t="n">
+        <v>45945158.82</v>
+      </c>
+      <c r="CZ13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -12857,7 +12977,10 @@
       <c r="CX14" s="4" t="n">
         <v>83428332.73999999</v>
       </c>
-      <c r="CY14" s="4" t="n"/>
+      <c r="CY14" s="4" t="n">
+        <v>72126498.09</v>
+      </c>
+      <c r="CZ14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -13079,6 +13202,7 @@
       <c r="CY15" s="4" t="n">
         <v>65773620.6</v>
       </c>
+      <c r="CZ15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -13252,6 +13376,7 @@
       <c r="CY16" s="4" t="n">
         <v>5084736.37</v>
       </c>
+      <c r="CZ16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -13495,6 +13620,7 @@
       <c r="CY17" s="4" t="n">
         <v>77499289.81999999</v>
       </c>
+      <c r="CZ17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -13608,12 +13734,15 @@
         <v>10301006.7</v>
       </c>
       <c r="CW18" s="4" t="n">
-        <v>26559675.22</v>
+        <v>20757549.6</v>
       </c>
       <c r="CX18" s="4" t="n">
-        <v>32508228.02</v>
-      </c>
-      <c r="CY18" s="4" t="n"/>
+        <v>20284823.76</v>
+      </c>
+      <c r="CY18" s="4" t="n">
+        <v>29356840.37</v>
+      </c>
+      <c r="CZ18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -13907,6 +14036,7 @@
       <c r="CY19" s="4" t="n">
         <v>1935113.39</v>
       </c>
+      <c r="CZ19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -14056,6 +14186,7 @@
       <c r="CY20" s="4" t="n">
         <v>477188.5</v>
       </c>
+      <c r="CZ20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -14223,6 +14354,7 @@
       <c r="CY21" s="4" t="n">
         <v>64318908</v>
       </c>
+      <c r="CZ21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -14404,6 +14536,7 @@
       <c r="CY22" s="4" t="n">
         <v>523246.02</v>
       </c>
+      <c r="CZ22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -14673,6 +14806,7 @@
       <c r="CY23" s="4" t="n">
         <v>7986249</v>
       </c>
+      <c r="CZ23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -14976,6 +15110,9 @@
       <c r="CY24" s="4" t="n">
         <v>83228511</v>
       </c>
+      <c r="CZ24" s="4" t="n">
+        <v>83228511</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -15284,7 +15421,10 @@
       <c r="CX25" s="4" t="n">
         <v>78680000</v>
       </c>
-      <c r="CY25" s="4" t="n"/>
+      <c r="CY25" s="4" t="n">
+        <v>72709000</v>
+      </c>
+      <c r="CZ25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -15504,6 +15644,7 @@
       <c r="CY26" s="4" t="n">
         <v>204161822</v>
       </c>
+      <c r="CZ26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -15685,18 +15826,19 @@
         <v>137671838</v>
       </c>
       <c r="CU27" s="4" t="n">
-        <v>99478687</v>
+        <v>92421083</v>
       </c>
       <c r="CV27" s="4" t="n">
-        <v>72604362</v>
+        <v>36389808</v>
       </c>
       <c r="CW27" s="4" t="n">
-        <v>54851275</v>
+        <v>25286642</v>
       </c>
       <c r="CX27" s="4" t="n">
-        <v>89183735</v>
+        <v>88959455</v>
       </c>
       <c r="CY27" s="4" t="n"/>
+      <c r="CZ27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -15962,6 +16104,7 @@
       <c r="CY28" s="4" t="n">
         <v>9809562</v>
       </c>
+      <c r="CZ28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -15997,13 +16140,13 @@
         <v>1319295.51</v>
       </c>
       <c r="Q29" s="4" t="n">
-        <v>4174942.33</v>
+        <v>4282039.28</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>3349728.75</v>
+        <v>3440319.04</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>2182069.74</v>
+        <v>2150006.32</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>2797949.4</v>
@@ -16257,6 +16400,7 @@
       <c r="CY29" s="4" t="n">
         <v>67649649.97</v>
       </c>
+      <c r="CZ29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -16546,6 +16690,7 @@
       </c>
       <c r="CX30" s="4" t="n"/>
       <c r="CY30" s="4" t="n"/>
+      <c r="CZ30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -16726,7 +16871,10 @@
       <c r="CX31" s="4" t="n">
         <v>116694.63</v>
       </c>
-      <c r="CY31" s="4" t="n"/>
+      <c r="CY31" s="4" t="n">
+        <v>15407.74</v>
+      </c>
+      <c r="CZ31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -16973,6 +17121,9 @@
       </c>
       <c r="CY32" s="4" t="n">
         <v>44303833</v>
+      </c>
+      <c r="CZ32" s="4" t="n">
+        <v>45612925.8</v>
       </c>
     </row>
     <row r="33">
@@ -17215,6 +17366,7 @@
         <v>69671591</v>
       </c>
       <c r="CY33" s="4" t="n"/>
+      <c r="CZ33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -17386,6 +17538,7 @@
       <c r="CY34" s="4" t="n">
         <v>1955300</v>
       </c>
+      <c r="CZ34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -17642,6 +17795,9 @@
       </c>
       <c r="CY35" s="4" t="n">
         <v>4718609.7</v>
+      </c>
+      <c r="CZ35" s="4" t="n">
+        <v>789081.05</v>
       </c>
     </row>
     <row r="36">
@@ -17699,26 +17855,54 @@
       <c r="AR36" s="4" t="n"/>
       <c r="AS36" s="4" t="n"/>
       <c r="AT36" s="4" t="n"/>
-      <c r="AU36" s="4" t="n"/>
-      <c r="AV36" s="4" t="n"/>
-      <c r="AW36" s="4" t="n"/>
+      <c r="AU36" s="4" t="n">
+        <v>955466.4</v>
+      </c>
+      <c r="AV36" s="4" t="n">
+        <v>881200.05</v>
+      </c>
+      <c r="AW36" s="4" t="n">
+        <v>1363696.28</v>
+      </c>
       <c r="AX36" s="4" t="n">
         <v>813504.21</v>
       </c>
-      <c r="AY36" s="4" t="n"/>
+      <c r="AY36" s="4" t="n">
+        <v>1098459.68</v>
+      </c>
       <c r="AZ36" s="4" t="n">
         <v>722630.77</v>
       </c>
-      <c r="BA36" s="4" t="n"/>
-      <c r="BB36" s="4" t="n"/>
-      <c r="BC36" s="4" t="n"/>
-      <c r="BD36" s="4" t="n"/>
-      <c r="BE36" s="4" t="n"/>
-      <c r="BF36" s="4" t="n"/>
-      <c r="BG36" s="4" t="n"/>
-      <c r="BH36" s="4" t="n"/>
-      <c r="BI36" s="4" t="n"/>
-      <c r="BJ36" s="4" t="n"/>
+      <c r="BA36" s="4" t="n">
+        <v>1101235.65</v>
+      </c>
+      <c r="BB36" s="4" t="n">
+        <v>1007796.24</v>
+      </c>
+      <c r="BC36" s="4" t="n">
+        <v>1011713.98</v>
+      </c>
+      <c r="BD36" s="4" t="n">
+        <v>673268.5</v>
+      </c>
+      <c r="BE36" s="4" t="n">
+        <v>680740.26</v>
+      </c>
+      <c r="BF36" s="4" t="n">
+        <v>1237814.86</v>
+      </c>
+      <c r="BG36" s="4" t="n">
+        <v>1932518.97</v>
+      </c>
+      <c r="BH36" s="4" t="n">
+        <v>2039620.37</v>
+      </c>
+      <c r="BI36" s="4" t="n">
+        <v>1478158.33</v>
+      </c>
+      <c r="BJ36" s="4" t="n">
+        <v>1803272.49</v>
+      </c>
       <c r="BK36" s="4" t="n">
         <v>1587273.19</v>
       </c>
@@ -17842,6 +18026,7 @@
       <c r="CY36" s="4" t="n">
         <v>1977424.41</v>
       </c>
+      <c r="CZ36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -17897,13 +18082,13 @@
         <v>51733851.59</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>74814284.97</v>
+        <v>74921381.92</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>50249420.15</v>
+        <v>50340010.44</v>
       </c>
       <c r="S37" s="6" t="n">
-        <v>31076585.86</v>
+        <v>31044522.44</v>
       </c>
       <c r="T37" s="6" t="n">
         <v>32068304.72</v>
@@ -17987,52 +18172,52 @@
         <v>246762904.19</v>
       </c>
       <c r="AU37" s="6" t="n">
-        <v>449126820.73</v>
+        <v>450082287.13</v>
       </c>
       <c r="AV37" s="6" t="n">
-        <v>460213605.24</v>
+        <v>461094805.29</v>
       </c>
       <c r="AW37" s="6" t="n">
-        <v>730204937.89</v>
+        <v>731568634.17</v>
       </c>
       <c r="AX37" s="6" t="n">
         <v>374225554.89</v>
       </c>
       <c r="AY37" s="6" t="n">
-        <v>647110766.54</v>
+        <v>648209226.22</v>
       </c>
       <c r="AZ37" s="6" t="n">
         <v>403941757.97</v>
       </c>
       <c r="BA37" s="6" t="n">
-        <v>614678489.33</v>
+        <v>615779724.98</v>
       </c>
       <c r="BB37" s="6" t="n">
-        <v>532981184.21</v>
+        <v>533988980.45</v>
       </c>
       <c r="BC37" s="6" t="n">
-        <v>595808316.13</v>
+        <v>596820030.11</v>
       </c>
       <c r="BD37" s="6" t="n">
-        <v>332937017.57</v>
+        <v>333610286.07</v>
       </c>
       <c r="BE37" s="6" t="n">
-        <v>417897885.75</v>
+        <v>418578626.01</v>
       </c>
       <c r="BF37" s="6" t="n">
-        <v>514391645.37</v>
+        <v>515629460.23</v>
       </c>
       <c r="BG37" s="6" t="n">
-        <v>916688845.86</v>
+        <v>918621364.83</v>
       </c>
       <c r="BH37" s="6" t="n">
-        <v>850689696.85</v>
+        <v>852729317.22</v>
       </c>
       <c r="BI37" s="6" t="n">
-        <v>772722476.4</v>
+        <v>774200634.73</v>
       </c>
       <c r="BJ37" s="6" t="n">
-        <v>890499263.16</v>
+        <v>892302535.65</v>
       </c>
       <c r="BK37" s="6" t="n">
         <v>1030639828.64</v>
@@ -18143,23 +18328,26 @@
         <v>1819377136.04</v>
       </c>
       <c r="CU37" s="6" t="n">
-        <v>1642580965.3</v>
+        <v>1635523361.3</v>
       </c>
       <c r="CV37" s="6" t="n">
-        <v>1189939194.79</v>
+        <v>1153724640.79</v>
       </c>
       <c r="CW37" s="6" t="n">
-        <v>1405750015.25</v>
+        <v>1370383256.63</v>
       </c>
       <c r="CX37" s="6" t="n">
-        <v>1506916269.24</v>
+        <v>1521655969.98</v>
       </c>
       <c r="CY37" s="6" t="n">
-        <v>764954248.28</v>
+        <v>1056260121.71</v>
+      </c>
+      <c r="CZ37" s="6" t="n">
+        <v>129630517.85</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CY36"/>
+  <autoFilter ref="A1:CZ36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18170,7 +18358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CY37"/>
+  <dimension ref="A1:CZ37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -18276,6 +18464,7 @@
     <col width="10" customWidth="1" min="101" max="101"/>
     <col width="10" customWidth="1" min="102" max="102"/>
     <col width="10" customWidth="1" min="103" max="103"/>
+    <col width="10" customWidth="1" min="104" max="104"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -18792,6 +18981,11 @@
       <c r="CY1" s="1" t="inlineStr">
         <is>
           <t>May 2026</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
         </is>
       </c>
     </row>
@@ -19049,6 +19243,7 @@
       <c r="CY2" s="7" t="n">
         <v>0.1</v>
       </c>
+      <c r="CZ2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -19272,6 +19467,7 @@
         <v>0.11205007465145</v>
       </c>
       <c r="CY3" s="7" t="n"/>
+      <c r="CZ3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -19526,7 +19722,10 @@
       <c r="CX4" s="7" t="n">
         <v>0.09567033221176095</v>
       </c>
-      <c r="CY4" s="7" t="n"/>
+      <c r="CY4" s="7" t="n">
+        <v>0.09519316724154857</v>
+      </c>
+      <c r="CZ4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -19752,6 +19951,7 @@
       <c r="CY5" s="7" t="n">
         <v>0.1023440773981386</v>
       </c>
+      <c r="CZ5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -20001,6 +20201,7 @@
       <c r="CY6" s="7" t="n">
         <v>0.1142111411492929</v>
       </c>
+      <c r="CZ6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -20136,6 +20337,7 @@
       <c r="CY7" s="7" t="n">
         <v>0.1115726549672448</v>
       </c>
+      <c r="CZ7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -20411,6 +20613,7 @@
       <c r="CY8" s="7" t="n">
         <v>0.1087623367597327</v>
       </c>
+      <c r="CZ8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -20668,6 +20871,7 @@
         <v>0.1039112064561212</v>
       </c>
       <c r="CY9" s="7" t="n"/>
+      <c r="CZ9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -20943,6 +21147,7 @@
       <c r="CY10" s="7" t="n">
         <v>0.1171592548945845</v>
       </c>
+      <c r="CZ10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -21132,6 +21337,7 @@
       <c r="CY11" s="7" t="n">
         <v>0.07339594087827053</v>
       </c>
+      <c r="CZ11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -21305,8 +21511,13 @@
       <c r="CW12" s="7" t="n">
         <v>0.09634772120452796</v>
       </c>
-      <c r="CX12" s="7" t="n"/>
-      <c r="CY12" s="7" t="n"/>
+      <c r="CX12" s="7" t="n">
+        <v>0.1181744825111545</v>
+      </c>
+      <c r="CY12" s="7" t="n">
+        <v>0.1101643233416123</v>
+      </c>
+      <c r="CZ12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -21527,7 +21738,10 @@
       <c r="CX13" s="7" t="n">
         <v>0.1412824578042649</v>
       </c>
-      <c r="CY13" s="7" t="n"/>
+      <c r="CY13" s="7" t="n">
+        <v>0.1444932776539814</v>
+      </c>
+      <c r="CZ13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -21720,7 +21934,10 @@
       <c r="CX14" s="7" t="n">
         <v>0.12298125459198</v>
       </c>
-      <c r="CY14" s="7" t="n"/>
+      <c r="CY14" s="7" t="n">
+        <v>0.1141044039346676</v>
+      </c>
+      <c r="CZ14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -21942,6 +22159,7 @@
       <c r="CY15" s="7" t="n">
         <v>0.1228459740501489</v>
       </c>
+      <c r="CZ15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -22115,6 +22333,7 @@
       <c r="CY16" s="7" t="n">
         <v>0.1241071980111299</v>
       </c>
+      <c r="CZ16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -22358,6 +22577,7 @@
       <c r="CY17" s="7" t="n">
         <v>0.1667381040352044</v>
       </c>
+      <c r="CZ17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -22471,12 +22691,15 @@
         <v>0.03718702247489727</v>
       </c>
       <c r="CW18" s="7" t="n">
-        <v>0.08064133786072113</v>
+        <v>0.0630247379378262</v>
       </c>
       <c r="CX18" s="7" t="n">
-        <v>0.1189044701197626</v>
-      </c>
-      <c r="CY18" s="7" t="n"/>
+        <v>0.07419525355770439</v>
+      </c>
+      <c r="CY18" s="7" t="n">
+        <v>0.1145119719578884</v>
+      </c>
+      <c r="CZ18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -22770,6 +22993,7 @@
       <c r="CY19" s="7" t="n">
         <v>0.1118688610403673</v>
       </c>
+      <c r="CZ19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -22919,6 +23143,7 @@
       <c r="CY20" s="7" t="n">
         <v>0.0991167759601546</v>
       </c>
+      <c r="CZ20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -23086,6 +23311,7 @@
       <c r="CY21" s="7" t="n">
         <v>0.1112648499990031</v>
       </c>
+      <c r="CZ21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -23199,6 +23425,7 @@
       <c r="CW22" s="7" t="n"/>
       <c r="CX22" s="7" t="n"/>
       <c r="CY22" s="7" t="n"/>
+      <c r="CZ22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -23468,6 +23695,7 @@
       <c r="CY23" s="7" t="n">
         <v>0.1310956165789779</v>
       </c>
+      <c r="CZ23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -23759,6 +23987,9 @@
       <c r="CY24" s="7" t="n">
         <v>0.09116943367707987</v>
       </c>
+      <c r="CZ24" s="7" t="n">
+        <v>0.09116943367707987</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -24067,7 +24298,10 @@
       <c r="CX25" s="7" t="n">
         <v>0.08526896551698936</v>
       </c>
-      <c r="CY25" s="7" t="n"/>
+      <c r="CY25" s="7" t="n">
+        <v>0.0760878828026382</v>
+      </c>
+      <c r="CZ25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -24287,6 +24521,7 @@
       <c r="CY26" s="7" t="n">
         <v>0.09572602909576347</v>
       </c>
+      <c r="CZ26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -24468,18 +24703,19 @@
         <v>0.1444669358188859</v>
       </c>
       <c r="CU27" s="7" t="n">
-        <v>0.1070619558894809</v>
+        <v>0.1137334235246944</v>
       </c>
       <c r="CV27" s="7" t="n">
-        <v>0.09469252800564766</v>
+        <v>0.1084273813733606</v>
       </c>
       <c r="CW27" s="7" t="n">
-        <v>0.0827250256916692</v>
+        <v>0.0716344810344212</v>
       </c>
       <c r="CX27" s="7" t="n">
-        <v>0.1114603880534236</v>
+        <v>0.1115102294810222</v>
       </c>
       <c r="CY27" s="7" t="n"/>
+      <c r="CZ27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -24745,6 +24981,7 @@
       <c r="CY28" s="7" t="n">
         <v>0.126391937251654</v>
       </c>
+      <c r="CZ28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -24780,13 +25017,13 @@
         <v>0.05649317744522721</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>0.1279651989019281</v>
+        <v>0.1212913513271294</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.1170852356376454</v>
+        <v>0.1192553212336825</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>0.07790406015044295</v>
+        <v>0.07521833838410455</v>
       </c>
       <c r="T29" s="7" t="n">
         <v>0.07122728049738432</v>
@@ -25040,6 +25277,7 @@
       <c r="CY29" s="7" t="n">
         <v>0.113588113097101</v>
       </c>
+      <c r="CZ29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -25329,6 +25567,7 @@
       </c>
       <c r="CX30" s="7" t="n"/>
       <c r="CY30" s="7" t="n"/>
+      <c r="CZ30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -25509,7 +25748,10 @@
       <c r="CX31" s="7" t="n">
         <v>0.1955063273919013</v>
       </c>
-      <c r="CY31" s="7" t="n"/>
+      <c r="CY31" s="7" t="n">
+        <v>0.03137152586505623</v>
+      </c>
+      <c r="CZ31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -25755,6 +25997,9 @@
         <v>0.1</v>
       </c>
       <c r="CY32" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="CZ32" s="7" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -25998,6 +26243,7 @@
         <v>0.1134913927882739</v>
       </c>
       <c r="CY33" s="7" t="n"/>
+      <c r="CZ33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -26169,6 +26415,7 @@
       <c r="CY34" s="7" t="n">
         <v>0.1397977426307328</v>
       </c>
+      <c r="CZ34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -26425,6 +26672,9 @@
       </c>
       <c r="CY35" s="7" t="n">
         <v>0.1431447679849384</v>
+      </c>
+      <c r="CZ35" s="7" t="n">
+        <v>0.1490564053372549</v>
       </c>
     </row>
     <row r="36">
@@ -26482,26 +26732,54 @@
       <c r="AR36" s="7" t="n"/>
       <c r="AS36" s="7" t="n"/>
       <c r="AT36" s="7" t="n"/>
-      <c r="AU36" s="7" t="n"/>
-      <c r="AV36" s="7" t="n"/>
-      <c r="AW36" s="7" t="n"/>
+      <c r="AU36" s="7" t="n">
+        <v>0.1531428771495591</v>
+      </c>
+      <c r="AV36" s="7" t="n">
+        <v>0.08123413505360402</v>
+      </c>
+      <c r="AW36" s="7" t="n">
+        <v>0.1242773375453754</v>
+      </c>
       <c r="AX36" s="7" t="n">
         <v>0.06621924692540988</v>
       </c>
-      <c r="AY36" s="7" t="n"/>
+      <c r="AY36" s="7" t="n">
+        <v>0.0785869624763614</v>
+      </c>
       <c r="AZ36" s="7" t="n">
         <v>0.0701474074805625</v>
       </c>
-      <c r="BA36" s="7" t="n"/>
-      <c r="BB36" s="7" t="n"/>
-      <c r="BC36" s="7" t="n"/>
-      <c r="BD36" s="7" t="n"/>
-      <c r="BE36" s="7" t="n"/>
-      <c r="BF36" s="7" t="n"/>
-      <c r="BG36" s="7" t="n"/>
-      <c r="BH36" s="7" t="n"/>
-      <c r="BI36" s="7" t="n"/>
-      <c r="BJ36" s="7" t="n"/>
+      <c r="BA36" s="7" t="n">
+        <v>0.0866777657998367</v>
+      </c>
+      <c r="BB36" s="7" t="n">
+        <v>0.1008207600799617</v>
+      </c>
+      <c r="BC36" s="7" t="n">
+        <v>0.1083108894224949</v>
+      </c>
+      <c r="BD36" s="7" t="n">
+        <v>0.09194074504580274</v>
+      </c>
+      <c r="BE36" s="7" t="n">
+        <v>0.09394247157555458</v>
+      </c>
+      <c r="BF36" s="7" t="n">
+        <v>0.1126217563001194</v>
+      </c>
+      <c r="BG36" s="7" t="n">
+        <v>0.1423568551085393</v>
+      </c>
+      <c r="BH36" s="7" t="n">
+        <v>0.1180655848016577</v>
+      </c>
+      <c r="BI36" s="7" t="n">
+        <v>0.0884972833112599</v>
+      </c>
+      <c r="BJ36" s="7" t="n">
+        <v>0.1195190690851537</v>
+      </c>
       <c r="BK36" s="7" t="n">
         <v>0.1106935138094091</v>
       </c>
@@ -26625,6 +26903,7 @@
       <c r="CY36" s="7" t="n">
         <v>0.1171026784762089</v>
       </c>
+      <c r="CZ36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -26680,13 +26959,13 @@
         <v>0.06099628568055292</v>
       </c>
       <c r="Q37" s="8" t="n">
-        <v>0.0707240832789425</v>
+        <v>0.0706464678147662</v>
       </c>
       <c r="R37" s="8" t="n">
-        <v>0.07112457818874983</v>
+        <v>0.07122870362153849</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>0.04435272756899608</v>
+        <v>0.04427070958576353</v>
       </c>
       <c r="T37" s="8" t="n">
         <v>0.04825857578193215</v>
@@ -26770,52 +27049,52 @@
         <v>0.07171241879256757</v>
       </c>
       <c r="AU37" s="8" t="n">
-        <v>0.07795815109262946</v>
+        <v>0.07803948482659237</v>
       </c>
       <c r="AV37" s="8" t="n">
-        <v>0.05790181194202801</v>
+        <v>0.05793361246886212</v>
       </c>
       <c r="AW37" s="8" t="n">
-        <v>0.09315452402467632</v>
+        <v>0.09319803073284715</v>
       </c>
       <c r="AX37" s="8" t="n">
         <v>0.04785669580290552</v>
       </c>
       <c r="AY37" s="8" t="n">
-        <v>0.06320462507594175</v>
+        <v>0.06322559677802361</v>
       </c>
       <c r="AZ37" s="8" t="n">
         <v>0.04911285264517534</v>
       </c>
       <c r="BA37" s="8" t="n">
-        <v>0.06428249391828039</v>
+        <v>0.06431221036948731</v>
       </c>
       <c r="BB37" s="8" t="n">
-        <v>0.06898998731461757</v>
+        <v>0.06903111957447489</v>
       </c>
       <c r="BC37" s="8" t="n">
-        <v>0.08753185860049097</v>
+        <v>0.08756033433513473</v>
       </c>
       <c r="BD37" s="8" t="n">
-        <v>0.06341791159038755</v>
+        <v>0.06345764148721401</v>
       </c>
       <c r="BE37" s="8" t="n">
-        <v>0.08800013863140706</v>
+        <v>0.08800919235899157</v>
       </c>
       <c r="BF37" s="8" t="n">
-        <v>0.1007865932830495</v>
+        <v>0.1008120253851331</v>
       </c>
       <c r="BG37" s="8" t="n">
-        <v>0.1138511428527034</v>
+        <v>0.113899122949039</v>
       </c>
       <c r="BH37" s="8" t="n">
-        <v>0.08610315363062228</v>
+        <v>0.08615894345497513</v>
       </c>
       <c r="BI37" s="8" t="n">
-        <v>0.07625033738895888</v>
+        <v>0.07627048955938683</v>
       </c>
       <c r="BJ37" s="8" t="n">
-        <v>0.0925495425306974</v>
+        <v>0.0925917663700089</v>
       </c>
       <c r="BK37" s="8" t="n">
         <v>0.08974587683132104</v>
@@ -26926,23 +27205,26 @@
         <v>0.1109596810864313</v>
       </c>
       <c r="CU37" s="8" t="n">
-        <v>0.1008994489862095</v>
+        <v>0.1011904266888519</v>
       </c>
       <c r="CV37" s="8" t="n">
-        <v>0.09104890611472208</v>
+        <v>0.09128935080613101</v>
       </c>
       <c r="CW37" s="8" t="n">
-        <v>0.09107102435950182</v>
+        <v>0.0905996888957581</v>
       </c>
       <c r="CX37" s="8" t="n">
-        <v>0.1111077684080403</v>
+        <v>0.110342109670582</v>
       </c>
       <c r="CY37" s="8" t="n">
-        <v>0.1077101386590889</v>
+        <v>0.1058999583441599</v>
+      </c>
+      <c r="CZ37" s="8" t="n">
+        <v>0.09432322363505194</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CY36"/>
+  <autoFilter ref="A1:CZ36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26976,7 +27258,7 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>2026-06-18 16:56 UTC</t>
+          <t>2026-07-08 17:37 UTC</t>
         </is>
       </c>
     </row>
@@ -26988,7 +27270,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Jan 2018 – May 2026  (101 monthly columns, 35 states + US total)</t>
+          <t>Jan 2018 – Jun 2026  (102 monthly columns, 35 states + US total)</t>
         </is>
       </c>
     </row>

</xml_diff>